<commit_message>
docs: enumerate every templated endpoint set
Expands the four places a {placeholder} still stood in for a real list:
- Caltrans CCTV: 12 district URLs (D01-D12)
- Caltrans CMS: 12 district URLs
- ARNOLD: 48 per-state FeatureServers, vintage 2019, own tab/section
- NHTSA FARS: the 5 year files actually fetched (2021-2025)

192 URLs in the workbook, 195 on the page. The only braces left are
genuine per-request parameters that cannot be enumerated: OSRM
coordinates, TomTom bbox, an NWS alert id, a Twilio account sid, and the
IBI/511 pagination offset.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KU6vCHVwj8n3HqfggcJ2CP
</commit_message>
<xml_diff>
--- a/docs/Consumed_APIs_for_MITRE.xlsx
+++ b/docs/Consumed_APIs_for_MITRE.xlsx
@@ -13,15 +13,17 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. DMS and device sources" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Milepost - LRS sources" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Reference and enrichment" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. Operational integrations" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. ARNOLD geometry services" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Operational integrations" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. Work-zone event feeds'!$A$1:$G$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Camera sources'!$A$1:$F$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. DMS and device sources'!$A$1:$I$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Camera sources'!$A$1:$F$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. DMS and device sources'!$A$1:$I$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. Milepost - LRS sources'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5. Reference and enrichment'!$A$1:$G$33</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6. Operational integrations'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5. Reference and enrichment'!$A$1:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6. ARNOLD geometry services'!$A$1:$D$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7. Operational integrations'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -105,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -129,9 +131,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -502,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -645,33 +644,45 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>31 endpoints: geometry, corroboration, safety, weather, freight, parking, routing, population, demand, grants.</t>
+          <t>36 endpoints: geometry, corroboration, safety, weather, freight, parking, routing, population, demand, grants.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>6. Operational integrations</t>
+          <t>6. ARNOLD geometry services</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>48 per-state FeatureServers, ARNOLD vintage 2019, enumerated individually.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>7. Operational integrations</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>7 services that ingest no data. Endpoints given where fixed; per-deployment where not.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Evidence grade</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Only sources carrying live telemetry can validate a work zone. PennDOT TSAMS and MaineDOT are static GIS asset inventories with no message field and no timestamp; their 853 records are ingested for coverage reporting but excluded from adjudication.</t>
         </is>
@@ -2118,7 +2129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2195,7 +2206,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>California — D01</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -2205,12 +2216,12 @@
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>https://cwwp2.dot.ca.gov/data/d{N}/cctv/cctvStatusD{NN}.json</t>
+          <t>https://cwwp2.dot.ca.gov/data/d1/cctv/cctvStatusD01.json</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>One request per Caltrans district, D01–D12</t>
+          <t>Caltrans district D01 of 12</t>
         </is>
       </c>
       <c r="F3" s="7" t="n">
@@ -2218,14 +2229,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
+      <c r="A4" s="5" t="inlineStr"/>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>California — D02</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -2235,143 +2242,117 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_Cameras/FeatureServer/0/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="5" t="n">
-        <v>1669</v>
-      </c>
+          <t>https://cwwp2.dot.ca.gov/data/d2/cctv/cctvStatusD02.json</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D02 of 12</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>GA</t>
-        </is>
-      </c>
+      <c r="A5" s="7" t="inlineStr"/>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>California — D03</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>https://511ga.org/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d3/cctv/cctvStatusD03.json</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="n">
-        <v>4043</v>
-      </c>
+          <t>Caltrans district D03 of 12</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
+      <c r="A6" s="5" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Idaho</t>
+          <t>California — D04</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>https://511.idaho.gov/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d4/cctv/cctvStatusD04.json</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>457</v>
-      </c>
+          <t>Caltrans district D04 of 12</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
+      <c r="A7" s="7" t="inlineStr"/>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Louisiana</t>
+          <t>California — D05</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>https://www.511la.org/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d5/cctv/cctvStatusD05.json</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>336</v>
-      </c>
+          <t>Caltrans district D05 of 12</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
+      <c r="A8" s="5" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Maine / New England</t>
+          <t>California — D06</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>https://newengland511.org/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d6/cctv/cctvStatusD06.json</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>405</v>
-      </c>
+          <t>Caltrans district D06 of 12</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>MN</t>
-        </is>
-      </c>
+      <c r="A9" s="7" t="inlineStr"/>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Minnesota</t>
+          <t>California — D07</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -2381,83 +2362,69 @@
       </c>
       <c r="D9" s="8" t="inlineStr">
         <is>
-          <t>https://mntg.carsprogram.org/cameras_v1/api/cameras</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="n">
-        <v>1528</v>
-      </c>
+          <t>https://cwwp2.dot.ca.gov/data/d7/cctv/cctvStatusD07.json</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Caltrans district D07 of 12</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
+      <c r="A10" s="5" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>North Carolina</t>
+          <t>California — D08</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>https://www.drivenc.gov/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d8/cctv/cctvStatusD08.json</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>1140</v>
-      </c>
+          <t>Caltrans district D08 of 12</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
+      <c r="A11" s="7" t="inlineStr"/>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>Nevada</t>
+          <t>California — D09</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>https://www.nvroads.com/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d9/cctv/cctvStatusD09.json</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>640</v>
-      </c>
+          <t>Caltrans district D09 of 12</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
+      <c r="A12" s="5" t="inlineStr"/>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>New York</t>
+          <t>California — D10</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -2467,83 +2434,73 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>https://511ny.org/api/getcameras?format=json</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr"/>
-      <c r="F12" s="5" t="n">
-        <v>1871</v>
-      </c>
+          <t>https://cwwp2.dot.ca.gov/data/d10/cctv/cctvStatusD10.json</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D10 of 12</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
+      <c r="A13" s="7" t="inlineStr"/>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Arizona</t>
+          <t>California — D11</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
         <is>
-          <t>https://az511.com/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d11/cctv/cctvStatusD11.json</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="n">
-        <v>644</v>
-      </c>
+          <t>Caltrans district D11 of 12</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>PA</t>
-        </is>
-      </c>
+      <c r="A14" s="5" t="inlineStr"/>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Pennsylvania</t>
+          <t>California — D12</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>https://www.511pa.com/List/GetData/Cameras</t>
+          <t>https://cwwp2.dot.ca.gov/data/d12/cctv/cctvStatusD12.json</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="n">
-        <v>1536</v>
-      </c>
+          <t>Caltrans district D12 of 12</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>TX</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Texas (Austin)</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -2553,64 +2510,382 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>https://data.austintexas.gov/resource/b4k4-adkb.json?$limit=2000</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Socrata; snapshots at https://cctv.austinmobility.io/image/{camera_id}.jpg</t>
-        </is>
-      </c>
+          <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_Cameras/FeatureServer/0/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
       <c r="F15" s="7" t="n">
-        <v>1005</v>
+        <v>1669</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Georgia</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>https://511ga.org/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>4043</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Idaho</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>https://511.idaho.gov/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Louisiana</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>https://www.511la.org/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Maine / New England</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>https://newengland511.org/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Minnesota</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>https://mntg.carsprogram.org/cameras_v1/api/cameras</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="n">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>https://www.drivenc.gov/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>1140</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.nvroads.com/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>https://511ny.org/api/getcameras?format=json</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+      <c r="F23" s="7" t="n">
+        <v>1871</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Arizona</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>https://az511.com/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>https://www.511pa.com/List/GetData/Cameras</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Texas (Austin)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>https://data.austintexas.gov/resource/b4k4-adkb.json?$limit=2000</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Socrata; snapshots at https://cctv.austinmobility.io/image/{camera_id}.jpg</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
           <t>UT</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Utah</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>https://www.udottraffic.utah.gov/List/GetData/Cameras</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>DataTables POST, paged: draw=1&amp;start={n}&amp;length=1000</t>
         </is>
       </c>
-      <c r="F16" s="5" t="n">
+      <c r="F27" s="7" t="n">
         <v>2075</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="9" t="inlineStr"/>
-      <c r="B17" s="9" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr"/>
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr"/>
-      <c r="D17" s="9" t="inlineStr"/>
-      <c r="E17" s="9" t="inlineStr"/>
-      <c r="F17" s="9" t="n">
+      <c r="C28" s="9" t="inlineStr"/>
+      <c r="D28" s="9" t="inlineStr"/>
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="F28" s="9" t="n">
         <v>21941</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F17"/>
+  <autoFilter ref="A1:F28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2621,7 +2896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2780,7 +3055,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>California</t>
+          <t>California — D01</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -2790,7 +3065,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>https://cwwp2.dot.ca.gov/data/d{N}/cms/cmsStatusD{NN}.json</t>
+          <t>https://cwwp2.dot.ca.gov/data/d1/cms/cmsStatusD01.json</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
@@ -2813,19 +3088,15 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>One request per Caltrans district, D01–D12.</t>
+          <t>Caltrans district D01 of 12; some districts intermittently 500 and are skipped.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
+      <c r="A5" s="7" t="inlineStr"/>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Florida</t>
+          <t>California — D02</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -2835,496 +3106,342 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_MessageBoard/FeatureServer/0/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>1138</v>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
+          <t>https://cwwp2.dot.ca.gov/data/d2/cms/cmsStatusD02.json</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="7" t="inlineStr"/>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>live telemetry</t>
-        </is>
-      </c>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Caltrans district D02 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr"/>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>California — D03</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d3/cms/cmsStatusD03.json</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Idaho</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>https://511.idaho.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D03 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>California — D04</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d4/cms/cmsStatusD04.json</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Caltrans district D04 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>California — D05</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d5/cms/cmsStatusD05.json</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>not ingested — key not set</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>ID_511_KEY</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Free 511 registration outstanding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>KY</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Kentucky</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>https://services2.arcgis.com/CcI36Pduqd0OR4W9/arcgis/rest/services/dmsSigns_2020/FeatureServer/0/query?where=dmsStatus%20%3D%20'Online'&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>88</v>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D05 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>California — D06</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d6/cms/cmsStatusD06.json</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>live telemetry</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Caltrans district D06 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>California — D07</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d7/cms/cmsStatusD07.json</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
+      <c r="H10" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>where-clause drops 2 Offline signs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>LA</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Louisiana</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>https://511la.org/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D07 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>California — D08</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d8/cms/cmsStatusD08.json</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Caltrans district D08 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>California — D09</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d9/cms/cmsStatusD09.json</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>not ingested — key not set</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>LA_511_KEY</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>Free 511 registration outstanding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>Maine</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>https://arcgisserver.maine.gov/arcgis/rest/services/mdot/MaineDOT_Dynamic/MapServer/111/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>101</v>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D09 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>California — D10</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d10/cms/cmsStatusD10.json</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>INVENTORY ONLY</t>
-        </is>
-      </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Caltrans district D10 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>California — D11</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d11/cms/cmsStatusD11.json</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>Static asset inventory: 101 Ver-Mac 'Trailer Mounted' changeable message signs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Maryland</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>https://chartimap1.sha.maryland.gov/arcgis/rest/services/CHART/DMS/MapServer/0/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>295</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Caltrans district D11 of 12; some districts intermittently 500 and are skipped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>California — D12</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>https://cwwp2.dot.ca.gov/data/d12/cms/cmsStatusD12.json</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>live telemetry</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>NV</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Nevada</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>https://www.nvroads.com/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>not ingested — key not set</t>
-        </is>
-      </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>NV_511_KEY</t>
-        </is>
-      </c>
-      <c r="I11" s="7" t="inlineStr">
-        <is>
-          <t>Free 511 registration outstanding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>NJ</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>New Jersey</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>https://511nj.org/api/getmessagesigns?key=&lt;KEY&gt;&amp;format=json</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>not ingested — key not set</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>NJ_511_KEY</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Free 511 registration outstanding.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>NM</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>New Mexico</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>https://servicev4.nmroads.com/RealMapWAR/GetMessageSigns</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>unreachable</t>
-        </is>
-      </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I13" s="7" t="inlineStr">
-        <is>
-          <t>TLS certificate expired.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>NY</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>https://511ny.org/api/getmessagesigns?format=json</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>925</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>live telemetry</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>Keyless CARS/OneStop path.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>North Carolina</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>https://www.drivenc.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>not ingested — key not set</t>
-        </is>
-      </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>NC_511_KEY</t>
-        </is>
-      </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>Free 511 registration outstanding.</t>
+          <t>Caltrans district D12 of 12; some districts intermittently 500 and are skipped.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>FL</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Oklahoma</t>
+          <t>Florida</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -3334,14 +3451,16 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>https://oktraffic.org/api/Devices?filter[include][]=address&amp;filter[include][]=deviceTypeName   +   GET https://oktraffic.org/api/DmsStatuses</t>
+          <t>https://gis.fdot.gov/arcgis/rest/services/DIVAS_MessageBoard/FeatureServer/0/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>167</v>
-      </c>
-      <c r="F16" s="5" t="n">
-        <v>7</v>
+        <v>1138</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
@@ -3353,21 +3472,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>ODOT models 'Trailer' as its own non-DMS class (deviceTypeNameId 9) — the towable boards. Two calls: device list + DMS statuses.</t>
-        </is>
-      </c>
+      <c r="I16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Pennsylvania</t>
+          <t>Idaho</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -3377,11 +3492,13 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>https://gis.penndot.gov/arcgis/rest/services/tsams/tsams/MapServer/17/query?where=DEVICE_STATUS%20%3D%20'Existing%2FStandby'&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>752</v>
+          <t>https://511.idaho.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
@@ -3390,29 +3507,29 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>INVENTORY ONLY</t>
+          <t>not ingested — key not set</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>ID_511_KEY</t>
         </is>
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>Static asset inventory (no message, no timestamp). where-clause excludes 185 Planned + 83 Programmed + 20 Down devices not in the field.</t>
+          <t>Free 511 registration outstanding.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>UT</t>
+          <t>KY</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Utah</t>
+          <t>Kentucky</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -3422,44 +3539,42 @@
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>https://www.udottraffic.utah.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
+          <t>https://services2.arcgis.com/CcI36Pduqd0OR4W9/arcgis/rest/services/dmsSigns_2020/FeatureServer/0/query?where=dmsStatus%20%3D%20'Online'&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>88</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="5" t="inlineStr">
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>live telemetry</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>not ingested — key not set</t>
-        </is>
-      </c>
-      <c r="H18" s="5" t="inlineStr">
-        <is>
-          <t>UT_511_KEY</t>
-        </is>
-      </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Free 511 registration outstanding.</t>
+          <t>where-clause drops 2 Offline signs.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>WA</t>
+          <t>LA</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Washington</t>
+          <t>Louisiana</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -3469,99 +3584,600 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>https://wzdx.wsdot.wa.gov/api/v4/DeviceFeed</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="F19" s="7" t="n">
-        <v>5</v>
+          <t>https://511la.org/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>live telemetry</t>
+          <t>not ingested — key not set</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>LA_511_KEY</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>The only source with a properly typed WZDx device_type field.</t>
+          <t>Free 511 registration outstanding.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Maine</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>https://arcgisserver.maine.gov/arcgis/rest/services/mdot/MaineDOT_Dynamic/MapServer/111/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>INVENTORY ONLY</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Static asset inventory: 101 Ver-Mac 'Trailer Mounted' changeable message signs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Maryland</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>https://chartimap1.sha.maryland.gov/arcgis/rest/services/CHART/DMS/MapServer/0/query?where=1%3D1&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>295</v>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>live telemetry</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Nevada</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>https://www.nvroads.com/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>not ingested — key not set</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>NV_511_KEY</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Free 511 registration outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>New Jersey</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>https://511nj.org/api/getmessagesigns?key=&lt;KEY&gt;&amp;format=json</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>not ingested — key not set</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>NJ_511_KEY</t>
+        </is>
+      </c>
+      <c r="I23" s="7" t="inlineStr">
+        <is>
+          <t>Free 511 registration outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>New Mexico</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>https://servicev4.nmroads.com/RealMapWAR/GetMessageSigns</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>unreachable</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>TLS certificate expired.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>https://511ny.org/api/getmessagesigns?format=json</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>925</v>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>live telemetry</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Keyless CARS/OneStop path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>https://www.drivenc.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>not ingested — key not set</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>NC_511_KEY</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Free 511 registration outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Oklahoma</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D27" s="8" t="inlineStr">
+        <is>
+          <t>https://oktraffic.org/api/Devices?filter[include][]=address&amp;filter[include][]=deviceTypeName   +   GET https://oktraffic.org/api/DmsStatuses</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>167</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>live telemetry</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>ODOT models 'Trailer' as its own non-DMS class (deviceTypeNameId 9) — the towable boards. Two calls: device list + DMS statuses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Pennsylvania</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>https://gis.penndot.gov/arcgis/rest/services/tsams/tsams/MapServer/17/query?where=DEVICE_STATUS%20%3D%20'Existing%2FStandby'&amp;outFields=*&amp;returnGeometry=true&amp;outSR=4326&amp;f=json&amp;resultRecordCount=4000</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>752</v>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>INVENTORY ONLY</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Static asset inventory (no message, no timestamp). where-clause excludes 185 Planned + 83 Programmed + 20 Down devices not in the field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Utah</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>https://www.udottraffic.utah.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>not ingested — key not set</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>UT_511_KEY</t>
+        </is>
+      </c>
+      <c r="I29" s="7" t="inlineStr">
+        <is>
+          <t>Free 511 registration outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>https://wzdx.wsdot.wa.gov/api/v4/DeviceFeed</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>live telemetry</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>The only source with a properly typed WZDx device_type field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
           <t>WI</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Wisconsin</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>https://511wi.gov/api/v2/get/messagesigns?key=&lt;KEY&gt;&amp;format=json</t>
         </is>
       </c>
-      <c r="E20" s="5" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F20" s="5" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>not ingested — key not set</t>
         </is>
       </c>
-      <c r="H20" s="5" t="inlineStr">
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>WI_511_KEY</t>
         </is>
       </c>
-      <c r="I20" s="5" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>Free 511 registration outstanding.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="9" t="inlineStr"/>
-      <c r="B21" s="9" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr"/>
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr"/>
-      <c r="D21" s="9" t="inlineStr"/>
-      <c r="E21" s="9" t="n">
+      <c r="C32" s="9" t="inlineStr"/>
+      <c r="D32" s="9" t="inlineStr"/>
+      <c r="E32" s="9" t="n">
         <v>4606</v>
       </c>
-      <c r="F21" s="9" t="n">
+      <c r="F32" s="9" t="n">
         <v>74</v>
       </c>
-      <c r="G21" s="9" t="inlineStr"/>
-      <c r="H21" s="9" t="inlineStr"/>
-      <c r="I21" s="9" t="inlineStr"/>
+      <c r="G32" s="9" t="inlineStr"/>
+      <c r="H32" s="9" t="inlineStr"/>
+      <c r="I32" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I21"/>
+  <autoFilter ref="A1:I32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4037,7 +4653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4109,7 +4725,7 @@
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_{STATE}_{YEAR}/FeatureServer/0/query</t>
+          <t>48 per-state services — all enumerated on the ARNOLD tab</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
@@ -4119,7 +4735,7 @@
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Route polylines by route id + milepost. {STATE} is the 2-letter code, {YEAR} the ARNOLD vintage.</t>
+          <t>Route polylines by route id + milepost. One FeatureServer per state, ARNOLD vintage 2019.</t>
         </is>
       </c>
     </row>
@@ -4469,7 +5085,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>FARS annual national CSV bundle</t>
+          <t>FARS 2021 national CSV bundle</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -4479,7 +5095,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/{YEAR}/National/FARS{YEAR}NationalCSV.zip</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2021/National/FARS2021NationalCSV.zip</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -4496,17 +5112,17 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Freight</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>FHWA / BTS</t>
+          <t>NHTSA</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>National Bridge Inventory (NTAD)</t>
+          <t>FARS 2022 national CSV bundle</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -4516,7 +5132,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/xOi1kZaI0eWDREZv/arcgis/rest/services/NTAD_National_Bridge_Inventory/FeatureServer/0/query</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2022/National/FARS2022NationalCSV.zip</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -4526,24 +5142,24 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>Vertical underclearance for OSOW; annotates zones with structures the route passes under.</t>
+          <t>Rolling 5-year window; the set refreshes monthly.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Freight</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>U.S. CBP</t>
+          <t>NHTSA</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Border wait times</t>
+          <t>FARS 2023 national CSV bundle</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -4553,7 +5169,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>https://bwt.cbp.gov/api/waittimes</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2023/National/FARS2023NationalCSV.zip</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -4563,24 +5179,24 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Crossing waits. CBP returns no coordinates; a local port_number lookup supplies them.</t>
+          <t>Rolling 5-year window; the set refreshes monthly.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Truck parking</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>MAASTO</t>
+          <t>NHTSA</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>TPIMS V2.2 static</t>
+          <t>FARS 2024 national CSV bundle</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -4590,7 +5206,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>https://truckparking.travelmidwest.com/TPIMS_Static.json</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2024/National/FARS2024NationalCSV.zip</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -4600,24 +5216,24 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>Site metadata: location, name, capacity, amenities.</t>
+          <t>Rolling 5-year window; the set refreshes monthly.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Truck parking</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>MAASTO</t>
+          <t>NHTSA</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>TPIMS V2.2 dynamic</t>
+          <t>FARS 2025 national CSV bundle</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -4627,7 +5243,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>https://truckparking.travelmidwest.com/TPIMS_Dynamic.json</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2025/National/FARS2025NationalCSV.zip</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -4637,24 +5253,24 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Live availability, joined to static on siteId.</t>
+          <t>Rolling 5-year window; the set refreshes monthly.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Truck parking</t>
+          <t>Freight</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>MnDOT</t>
+          <t>FHWA / BTS</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>IRIS TPIMS static</t>
+          <t>National Bridge Inventory (NTAD)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -4664,7 +5280,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>http://iris.dot.state.mn.us/iris/TPIMS_static</t>
+          <t>https://services.arcgis.com/xOi1kZaI0eWDREZv/arcgis/rest/services/NTAD_National_Bridge_Inventory/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -4674,24 +5290,24 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Minnesota parking sites.</t>
+          <t>Vertical underclearance for OSOW; annotates zones with structures the route passes under.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Truck parking</t>
+          <t>Freight</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>MnDOT</t>
+          <t>U.S. CBP</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>IRIS TPIMS dynamic</t>
+          <t>Border wait times</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -4701,7 +5317,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>http://iris.dot.state.mn.us/iris/TPIMS_dynamic</t>
+          <t>https://bwt.cbp.gov/api/waittimes</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -4711,7 +5327,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Minnesota live availability.</t>
+          <t>Crossing waits. CBP returns no coordinates; a local port_number lookup supplies them.</t>
         </is>
       </c>
     </row>
@@ -4723,12 +5339,12 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>TRIMARC (KY)</t>
+          <t>MAASTO</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>TPIMS static</t>
+          <t>TPIMS V2.2 static</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -4738,7 +5354,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>http://www.trimarc.org/dat/tpims/TPIMS_Static.json</t>
+          <t>https://truckparking.travelmidwest.com/TPIMS_Static.json</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -4748,7 +5364,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Kentucky parking sites.</t>
+          <t>Site metadata: location, name, capacity, amenities.</t>
         </is>
       </c>
     </row>
@@ -4760,12 +5376,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>TRIMARC (KY)</t>
+          <t>MAASTO</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>TPIMS dynamic</t>
+          <t>TPIMS V2.2 dynamic</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -4775,7 +5391,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>http://www.trimarc.org/dat/tpims/TPIMS_Dynamic.json</t>
+          <t>https://truckparking.travelmidwest.com/TPIMS_Dynamic.json</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -4785,24 +5401,24 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Kentucky live availability.</t>
+          <t>Live availability, joined to static on siteId.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>V2X</t>
+          <t>Truck parking</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>FHWA / BTS</t>
+          <t>MnDOT</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>RSU Deployment Locations (NTAD)</t>
+          <t>IRIS TPIMS static</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -4812,7 +5428,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>https://geo.dot.gov/server/rest/services/Hosted/RSU_Deployment_Locations_010726/FeatureServer/0/query</t>
+          <t>http://iris.dot.state.mn.us/iris/TPIMS_static</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -4822,24 +5438,24 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Roadside-unit inventory for the connected-vehicle layer.</t>
+          <t>Minnesota parking sites.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Routing</t>
+          <t>Truck parking</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Project OSRM</t>
+          <t>MnDOT</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Route service v1 (2-point)</t>
+          <t>IRIS TPIMS dynamic</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -4849,7 +5465,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>https://router.project-osrm.org/route/v1/driving/{lon1},{lat1};{lon2},{lat2}?overview=full&amp;geometries=geojson</t>
+          <t>http://iris.dot.state.mn.us/iris/TPIMS_dynamic</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -4859,24 +5475,24 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Detour geometry and travel time. Public demo server; results cached persistently in osrm_geometry_cache.</t>
+          <t>Minnesota live availability.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Routing</t>
+          <t>Truck parking</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Project OSRM</t>
+          <t>TRIMARC (KY)</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Route service v1 (via-point)</t>
+          <t>TPIMS static</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -4886,7 +5502,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>https://router.project-osrm.org/route/v1/driving/{sLon},{sLat};{vLon},{vLat};{eLon},{eLat}?overview=full&amp;geometries=geojson</t>
+          <t>http://www.trimarc.org/dat/tpims/TPIMS_Static.json</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -4896,24 +5512,24 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Diversion route forced through a via point.</t>
+          <t>Kentucky parking sites.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Truck parking</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>US Census Bureau</t>
+          <t>TRIMARC (KY)</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Decennial PL 94-171</t>
+          <t>TPIMS dynamic</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -4923,34 +5539,34 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>https://api.census.gov/data/2020/dec/pl</t>
+          <t>http://www.trimarc.org/dat/tpims/TPIMS_Dynamic.json</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>key required</t>
+          <t>open</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Block-level population for IPAWS geofence exposure.</t>
+          <t>Kentucky live availability.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>US Census Bureau</t>
+          <t>FHWA / BTS</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>TIGERweb current</t>
+          <t>RSU Deployment Locations (NTAD)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -4960,7 +5576,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>https://tigerweb.geo.census.gov/arcgis/rest/services/TIGERweb/tigerWMS_Current/MapServer</t>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/RSU_Deployment_Locations_010726/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -4970,34 +5586,34 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Urban-area boundaries for alert masking.</t>
+          <t>Roadside-unit inventory for the connected-vehicle layer.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Routing</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>Project OSRM</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Overpass API</t>
+          <t>Route service v1 (2-point)</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>https://overpass-api.de/api/interpreter</t>
+          <t>https://router.project-osrm.org/route/v1/driving/{lon1},{lat1};{lon2},{lat2}?overview=full&amp;geometries=geojson</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -5007,24 +5623,24 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>POI and road context. Fair-use.</t>
+          <t>Detour geometry and travel time. Public demo server; results cached persistently in osrm_geometry_cache.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Routing</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>Project OSRM</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Nominatim</t>
+          <t>Route service v1 (via-point)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -5034,7 +5650,7 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>https://nominatim.openstreetmap.org</t>
+          <t>https://router.project-osrm.org/route/v1/driving/{sLon},{sLat};{vLon},{vLat};{eLon},{eLat}?overview=full&amp;geometries=geojson</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
@@ -5044,7 +5660,7 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Place-name geocoding. Fair-use.</t>
+          <t>Diversion route forced through a via point.</t>
         </is>
       </c>
     </row>
@@ -5056,12 +5672,12 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Iowa DNR</t>
+          <t>US Census Bureau</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>ArcGIS services root</t>
+          <t>Decennial PL 94-171</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -5071,17 +5687,17 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>https://data.iowadnr.gov/arcgis/rest/services</t>
+          <t>https://api.census.gov/data/2020/dec/pl</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>key required</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Iowa land-cover context.</t>
+          <t>Block-level population for IPAWS geofence exposure.</t>
         </is>
       </c>
     </row>
@@ -5093,12 +5709,12 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Iowa DOT</t>
+          <t>US Census Bureau</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>ArcGIS services root</t>
+          <t>TIGERweb current</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -5108,7 +5724,7 @@
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>https://maps.iowadot.gov/arcgis/rest/services</t>
+          <t>https://tigerweb.geo.census.gov/arcgis/rest/services/TIGERweb/tigerWMS_Current/MapServer</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -5118,61 +5734,61 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Iowa base layers.</t>
+          <t>Urban-area boundaries for alert masking.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Demand</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Ticketmaster</t>
+          <t>OpenStreetMap</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Discovery API v2</t>
+          <t>Overpass API</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>https://app.ticketmaster.com/discovery/v2/events.json?apikey=&lt;KEY&gt;</t>
+          <t>https://overpass-api.de/api/interpreter</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>key required</t>
+          <t>open</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Event demand surges near the corridor. Key not yet set.</t>
+          <t>POI and road context. Fair-use.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Demand</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>PredictHQ</t>
+          <t>OpenStreetMap</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Events API v1</t>
+          <t>Nominatim</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -5182,44 +5798,44 @@
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>https://api.predicthq.com/v1/events/</t>
+          <t>https://nominatim.openstreetmap.org</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>key required</t>
+          <t>open</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Alternate demand-surge source.</t>
+          <t>Place-name geocoding. Fair-use.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Grants</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Grants.gov</t>
+          <t>Iowa DNR</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>search2</t>
+          <t>ArcGIS services root</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>https://api.grants.gov/v1/api/search2</t>
+          <t>https://data.iowadnr.gov/arcgis/rest/services</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -5229,54 +5845,1301 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Federal opportunities, filtered to an ITS / digital-infrastructure keyword set.</t>
+          <t>Iowa land-cover context.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
+          <t>Population</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Iowa DOT</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>ArcGIS services root</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>https://maps.iowadot.gov/arcgis/rest/services</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>Iowa base layers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Ticketmaster</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Discovery API v2</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="inlineStr">
+        <is>
+          <t>https://app.ticketmaster.com/discovery/v2/events.json?apikey=&lt;KEY&gt;</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>key required</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>Event demand surges near the corridor. Key not yet set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Demand</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>PredictHQ</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Events API v1</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>https://api.predicthq.com/v1/events/</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>key required</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>Alternate demand-surge source.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
           <t>Grants</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>Grants.gov</t>
         </is>
       </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>search2</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="E36" s="6" t="inlineStr">
+        <is>
+          <t>https://api.grants.gov/v1/api/search2</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>Federal opportunities, filtered to an ITS / digital-infrastructure keyword set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Grants</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Grants.gov</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>fetchOpportunity</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>https://api.grants.gov/v1/api/fetchOpportunity</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>open</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>Full detail for one opportunity.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G33"/>
+  <autoFilter ref="A1:G37"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="104" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Full endpoint URL</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_CA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_OR_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_WA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>AZ</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_AZ_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_CO_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_ID_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>MT</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MT_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>NV</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NV_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>NM</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NM_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C11" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_UT_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>WY</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_WY_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_OK_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_TX_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_IL_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_IN_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MI_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_OH_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_WI_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_IA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_KS_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MN_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MO_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_ND_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NE_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_SD_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>AL</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_AL_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_AR_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_FL_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_GA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_KY_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_LA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MS_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NC_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_SC_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>TN</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_TN_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_VA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>WV</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_WV_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>CT</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_CT_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>DE</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_DE_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_MD_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_ME_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>NH</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NH_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NJ_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_NY_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_PA_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>RI</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_RI_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>VT</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/ARNOLD_VT_2019/FeatureServer/0/query</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD vintage 2019</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D49"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5474,7 +7337,7 @@
       <c r="D9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>

</xml_diff>

<commit_message>
docs: explain each runtime parameter; drop two never-fetched URLs
Adds a Runtime parameters tab/section documenting the five values filled
in at call time — TomTom bbox tiles, the OSRM 2-point and via-point
coordinate lists, the IBI/511 pagination offset, and the Twilio account
sid — with the deriving code, governing constants, and the effect each
has on request volume.

Also corrects an overstatement: api.weather.gov/alerts/{alertId} and
grants.gov/search-grants were listed as consumed endpoints, but neither
is ever requested. Both are click-through permalinks constructed on
records the platform emits. They are now called out as not-fetched
rather than counted as APIs we pull.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KU6vCHVwj8n3HqfggcJ2CP
</commit_message>
<xml_diff>
--- a/docs/Consumed_APIs_for_MITRE.xlsx
+++ b/docs/Consumed_APIs_for_MITRE.xlsx
@@ -14,16 +14,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. Milepost - LRS sources" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Reference and enrichment" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. ARNOLD geometry services" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Operational integrations" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. Runtime parameters" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8. Operational integrations" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. Work-zone event feeds'!$A$1:$G$38</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2. Camera sources'!$A$1:$F$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3. DMS and device sources'!$A$1:$I$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'4. Milepost - LRS sources'!$A$1:$E$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5. Reference and enrichment'!$A$1:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'5. Reference and enrichment'!$A$1:$G$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'6. ARNOLD geometry services'!$A$1:$D$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7. Operational integrations'!$A$1:$D$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'7. Runtime parameters'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'8. Operational integrations'!$A$1:$D$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +63,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C1F1F"/>
     </font>
   </fonts>
   <fills count="4">
@@ -107,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -134,6 +140,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -501,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -644,7 +653,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>36 endpoints: geometry, corroboration, safety, weather, freight, parking, routing, population, demand, grants.</t>
+          <t>35 endpoints: geometry, corroboration, safety, weather, freight, parking, routing, population, demand, grants.</t>
         </is>
       </c>
     </row>
@@ -663,26 +672,38 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>7. Operational integrations</t>
+          <t>7. Runtime parameters</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>Every {braced} value that varies per request: what it is, the code that derives it, and what it costs in requests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>8. Operational integrations</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>7 services that ingest no data. Endpoints given where fixed; per-deployment where not.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
-      <c r="B17" s="2" t="inlineStr"/>
-    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Evidence grade</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Only sources carrying live telemetry can validate a work zone. PennDOT TSAMS and MaineDOT are static GIS asset inventories with no message field and no timestamp; their 853 records are ingested for coverage reporting but excluded from adjudication.</t>
         </is>
@@ -4653,7 +4674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5038,17 +5059,17 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>NOAA / NWS</t>
+          <t>NHTSA</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Single alert by id</t>
+          <t>FARS 2021 national CSV bundle</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -5058,7 +5079,7 @@
       </c>
       <c r="E11" s="8" t="inlineStr">
         <is>
-          <t>https://api.weather.gov/alerts/{alertId}</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2021/National/FARS2021NationalCSV.zip</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -5068,7 +5089,7 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Detail fetch for an alert already seen in the active list.</t>
+          <t>Work-zone (WRK_ZONE) and large-truck (BODY_TYP + MCARR_ID) crash history. Bulk files because the live CrashAPI 403s datacenter IPs.</t>
         </is>
       </c>
     </row>
@@ -5085,7 +5106,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>FARS 2021 national CSV bundle</t>
+          <t>FARS 2022 national CSV bundle</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
@@ -5095,7 +5116,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2021/National/FARS2021NationalCSV.zip</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2022/National/FARS2022NationalCSV.zip</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
@@ -5105,7 +5126,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Work-zone (WRK_ZONE) and large-truck (BODY_TYP + MCARR_ID) crash history. Bulk files because the live CrashAPI 403s datacenter IPs.</t>
+          <t>Rolling 5-year window; the set refreshes monthly.</t>
         </is>
       </c>
     </row>
@@ -5122,7 +5143,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>FARS 2022 national CSV bundle</t>
+          <t>FARS 2023 national CSV bundle</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -5132,7 +5153,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2022/National/FARS2022NationalCSV.zip</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2023/National/FARS2023NationalCSV.zip</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -5159,7 +5180,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>FARS 2023 national CSV bundle</t>
+          <t>FARS 2024 national CSV bundle</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -5169,7 +5190,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2023/National/FARS2023NationalCSV.zip</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2024/National/FARS2024NationalCSV.zip</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -5196,7 +5217,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>FARS 2024 national CSV bundle</t>
+          <t>FARS 2025 national CSV bundle</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -5206,7 +5227,7 @@
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2024/National/FARS2024NationalCSV.zip</t>
+          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2025/National/FARS2025NationalCSV.zip</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -5223,17 +5244,17 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Freight</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>NHTSA</t>
+          <t>FHWA / BTS</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>FARS 2025 national CSV bundle</t>
+          <t>National Bridge Inventory (NTAD)</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -5243,7 +5264,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>https://static.nhtsa.gov/nhtsa/downloads/FARS/2025/National/FARS2025NationalCSV.zip</t>
+          <t>https://services.arcgis.com/xOi1kZaI0eWDREZv/arcgis/rest/services/NTAD_National_Bridge_Inventory/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -5253,7 +5274,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Rolling 5-year window; the set refreshes monthly.</t>
+          <t>Vertical underclearance for OSOW; annotates zones with structures the route passes under.</t>
         </is>
       </c>
     </row>
@@ -5265,12 +5286,12 @@
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>FHWA / BTS</t>
+          <t>U.S. CBP</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>National Bridge Inventory (NTAD)</t>
+          <t>Border wait times</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -5280,7 +5301,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/xOi1kZaI0eWDREZv/arcgis/rest/services/NTAD_National_Bridge_Inventory/FeatureServer/0/query</t>
+          <t>https://bwt.cbp.gov/api/waittimes</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -5290,24 +5311,24 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Vertical underclearance for OSOW; annotates zones with structures the route passes under.</t>
+          <t>Crossing waits. CBP returns no coordinates; a local port_number lookup supplies them.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Freight</t>
+          <t>Truck parking</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>U.S. CBP</t>
+          <t>MAASTO</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Border wait times</t>
+          <t>TPIMS V2.2 static</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
@@ -5317,7 +5338,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>https://bwt.cbp.gov/api/waittimes</t>
+          <t>https://truckparking.travelmidwest.com/TPIMS_Static.json</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
@@ -5327,7 +5348,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Crossing waits. CBP returns no coordinates; a local port_number lookup supplies them.</t>
+          <t>Site metadata: location, name, capacity, amenities.</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5365,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>TPIMS V2.2 static</t>
+          <t>TPIMS V2.2 dynamic</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -5354,7 +5375,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t>https://truckparking.travelmidwest.com/TPIMS_Static.json</t>
+          <t>https://truckparking.travelmidwest.com/TPIMS_Dynamic.json</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
@@ -5364,7 +5385,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>Site metadata: location, name, capacity, amenities.</t>
+          <t>Live availability, joined to static on siteId.</t>
         </is>
       </c>
     </row>
@@ -5376,12 +5397,12 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>MAASTO</t>
+          <t>MnDOT</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>TPIMS V2.2 dynamic</t>
+          <t>IRIS TPIMS static</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -5391,7 +5412,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>https://truckparking.travelmidwest.com/TPIMS_Dynamic.json</t>
+          <t>http://iris.dot.state.mn.us/iris/TPIMS_static</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
@@ -5401,7 +5422,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Live availability, joined to static on siteId.</t>
+          <t>Minnesota parking sites.</t>
         </is>
       </c>
     </row>
@@ -5418,7 +5439,7 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>IRIS TPIMS static</t>
+          <t>IRIS TPIMS dynamic</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -5428,7 +5449,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t>http://iris.dot.state.mn.us/iris/TPIMS_static</t>
+          <t>http://iris.dot.state.mn.us/iris/TPIMS_dynamic</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
@@ -5438,7 +5459,7 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>Minnesota parking sites.</t>
+          <t>Minnesota live availability.</t>
         </is>
       </c>
     </row>
@@ -5450,12 +5471,12 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>MnDOT</t>
+          <t>TRIMARC (KY)</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>IRIS TPIMS dynamic</t>
+          <t>TPIMS static</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -5465,7 +5486,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>http://iris.dot.state.mn.us/iris/TPIMS_dynamic</t>
+          <t>http://www.trimarc.org/dat/tpims/TPIMS_Static.json</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
@@ -5475,7 +5496,7 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Minnesota live availability.</t>
+          <t>Kentucky parking sites.</t>
         </is>
       </c>
     </row>
@@ -5492,7 +5513,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>TPIMS static</t>
+          <t>TPIMS dynamic</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -5502,7 +5523,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t>http://www.trimarc.org/dat/tpims/TPIMS_Static.json</t>
+          <t>http://www.trimarc.org/dat/tpims/TPIMS_Dynamic.json</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
@@ -5512,24 +5533,24 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>Kentucky parking sites.</t>
+          <t>Kentucky live availability.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Truck parking</t>
+          <t>V2X</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>TRIMARC (KY)</t>
+          <t>FHWA / BTS</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>TPIMS dynamic</t>
+          <t>RSU Deployment Locations (NTAD)</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -5539,7 +5560,7 @@
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>http://www.trimarc.org/dat/tpims/TPIMS_Dynamic.json</t>
+          <t>https://geo.dot.gov/server/rest/services/Hosted/RSU_Deployment_Locations_010726/FeatureServer/0/query</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
@@ -5549,24 +5570,24 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Kentucky live availability.</t>
+          <t>Roadside-unit inventory for the connected-vehicle layer.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>V2X</t>
+          <t>Routing</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>FHWA / BTS</t>
+          <t>Project OSRM</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>RSU Deployment Locations (NTAD)</t>
+          <t>Route service v1 (2-point)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -5576,7 +5597,7 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>https://geo.dot.gov/server/rest/services/Hosted/RSU_Deployment_Locations_010726/FeatureServer/0/query</t>
+          <t>https://router.project-osrm.org/route/v1/driving/{lon1},{lat1};{lon2},{lat2}?overview=full&amp;geometries=geojson</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -5586,7 +5607,7 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>Roadside-unit inventory for the connected-vehicle layer.</t>
+          <t>Detour geometry and travel time. Public demo server; results cached persistently in osrm_geometry_cache.</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5624,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Route service v1 (2-point)</t>
+          <t>Route service v1 (via-point)</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -5613,7 +5634,7 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>https://router.project-osrm.org/route/v1/driving/{lon1},{lat1};{lon2},{lat2}?overview=full&amp;geometries=geojson</t>
+          <t>https://router.project-osrm.org/route/v1/driving/{sLon},{sLat};{vLon},{vLat};{eLon},{eLat}?overview=full&amp;geometries=geojson</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -5623,24 +5644,24 @@
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Detour geometry and travel time. Public demo server; results cached persistently in osrm_geometry_cache.</t>
+          <t>Diversion route forced through a via point.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>Routing</t>
+          <t>Population</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Project OSRM</t>
+          <t>US Census Bureau</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Route service v1 (via-point)</t>
+          <t>Decennial PL 94-171</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -5650,17 +5671,17 @@
       </c>
       <c r="E27" s="8" t="inlineStr">
         <is>
-          <t>https://router.project-osrm.org/route/v1/driving/{sLon},{sLat};{vLon},{vLat};{eLon},{eLat}?overview=full&amp;geometries=geojson</t>
+          <t>https://api.census.gov/data/2020/dec/pl</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>key required</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>Diversion route forced through a via point.</t>
+          <t>Block-level population for IPAWS geofence exposure.</t>
         </is>
       </c>
     </row>
@@ -5677,7 +5698,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Decennial PL 94-171</t>
+          <t>TIGERweb current</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -5687,17 +5708,17 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>https://api.census.gov/data/2020/dec/pl</t>
+          <t>https://tigerweb.geo.census.gov/arcgis/rest/services/TIGERweb/tigerWMS_Current/MapServer</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>key required</t>
+          <t>open</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Block-level population for IPAWS geofence exposure.</t>
+          <t>Urban-area boundaries for alert masking.</t>
         </is>
       </c>
     </row>
@@ -5709,22 +5730,22 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>US Census Bureau</t>
+          <t>OpenStreetMap</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>TIGERweb current</t>
+          <t>Overpass API</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E29" s="8" t="inlineStr">
         <is>
-          <t>https://tigerweb.geo.census.gov/arcgis/rest/services/TIGERweb/tigerWMS_Current/MapServer</t>
+          <t>https://overpass-api.de/api/interpreter</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -5734,7 +5755,7 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>Urban-area boundaries for alert masking.</t>
+          <t>POI and road context. Fair-use.</t>
         </is>
       </c>
     </row>
@@ -5751,17 +5772,17 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Overpass API</t>
+          <t>Nominatim</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>https://overpass-api.de/api/interpreter</t>
+          <t>https://nominatim.openstreetmap.org</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
@@ -5771,7 +5792,7 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>POI and road context. Fair-use.</t>
+          <t>Place-name geocoding. Fair-use.</t>
         </is>
       </c>
     </row>
@@ -5783,12 +5804,12 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>Iowa DNR</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Nominatim</t>
+          <t>ArcGIS services root</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -5798,7 +5819,7 @@
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>https://nominatim.openstreetmap.org</t>
+          <t>https://data.iowadnr.gov/arcgis/rest/services</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -5808,7 +5829,7 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>Place-name geocoding. Fair-use.</t>
+          <t>Iowa land-cover context.</t>
         </is>
       </c>
     </row>
@@ -5820,7 +5841,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Iowa DNR</t>
+          <t>Iowa DOT</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -5835,7 +5856,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>https://data.iowadnr.gov/arcgis/rest/services</t>
+          <t>https://maps.iowadot.gov/arcgis/rest/services</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -5845,24 +5866,24 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Iowa land-cover context.</t>
+          <t>Iowa base layers.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Population</t>
+          <t>Demand</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>Iowa DOT</t>
+          <t>Ticketmaster</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>ArcGIS services root</t>
+          <t>Discovery API v2</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -5872,17 +5893,17 @@
       </c>
       <c r="E33" s="8" t="inlineStr">
         <is>
-          <t>https://maps.iowadot.gov/arcgis/rest/services</t>
+          <t>https://app.ticketmaster.com/discovery/v2/events.json?apikey=&lt;KEY&gt;</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>key required</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>Iowa base layers.</t>
+          <t>Event demand surges near the corridor. Key not yet set.</t>
         </is>
       </c>
     </row>
@@ -5894,12 +5915,12 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>Ticketmaster</t>
+          <t>PredictHQ</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Discovery API v2</t>
+          <t>Events API v1</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -5909,7 +5930,7 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>https://app.ticketmaster.com/discovery/v2/events.json?apikey=&lt;KEY&gt;</t>
+          <t>https://api.predicthq.com/v1/events/</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -5919,44 +5940,44 @@
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Event demand surges near the corridor. Key not yet set.</t>
+          <t>Alternate demand-surge source.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Demand</t>
+          <t>Grants</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>PredictHQ</t>
+          <t>Grants.gov</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Events API v1</t>
+          <t>search2</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>https://api.predicthq.com/v1/events/</t>
+          <t>https://api.grants.gov/v1/api/search2</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
         <is>
-          <t>key required</t>
+          <t>open</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>Alternate demand-surge source.</t>
+          <t>Federal opportunities, filtered to an ITS / digital-infrastructure keyword set.</t>
         </is>
       </c>
     </row>
@@ -5973,7 +5994,7 @@
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>search2</t>
+          <t>fetchOpportunity</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -5983,7 +6004,7 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>https://api.grants.gov/v1/api/search2</t>
+          <t>https://api.grants.gov/v1/api/fetchOpportunity</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -5993,49 +6014,12 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Federal opportunities, filtered to an ITS / digital-infrastructure keyword set.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>Grants</t>
-        </is>
-      </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>Grants.gov</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
-        <is>
-          <t>fetchOpportunity</t>
-        </is>
-      </c>
-      <c r="D37" s="7" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="E37" s="8" t="inlineStr">
-        <is>
-          <t>https://api.grants.gov/v1/api/fetchOpportunity</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
           <t>Full detail for one opportunity.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G37"/>
+  <autoFilter ref="A1:G36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7145,6 +7129,317 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="86" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Used by</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>How it is derived (code)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Governing constants</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Effect on request volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>{minLon},{minLat},{maxLon},{maxLat}</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>TomTom Traffic Incident Details v5</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>A bounding-box tile. TomTom caps one bbox at 10,000 km², so a corridor cannot be queried in a single call — it is covered by a chain of tiles.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>services/tomtom-incidents.js has two tilers. corridorTiles() walks the corridor polyline accumulating points and, as soon as the next point would push the bounding box past maxAreaKm2, emits the box built so far and starts a new one at that point. pointsToTiles() instead buckets the active work-zone coordinates onto a coarse grid and emits one padded tile per OCCUPIED cell, so N clustered zones cost far fewer requests than one bbox per zone. Both pad in kilometres converted to degrees: dLat = padKm / 110.574 and dLon = padKm / (111.320 × cos(midLat)).</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>corridorTiles: maxAreaKm2 9500 (under TomTom's 10,000), padKm 10, maxTiles 90. pointsToTiles: cellDeg 0.8 (≈7,100 km² even at Florida's latitude), padKm 3, maxTiles 220.</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>One request per tile per poll. Corridor tiles are deduped on a ~0.25° grid so overlapping directions and corridors do not pay twice. Self-capped by DAILY_BUDGET (default 2500/day, TOMTOM_DAILY_BUDGET to override); corridor TTL 45 min, zone TTL 6 h.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>{lon1},{lat1};{lon2},{lat2}</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>OSRM route service v1</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>The work zone's own two endpoints — the start and end coordinate of the event being snapped to the road network.</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>backend_proxy_server.js snapToRoad(lat1, lng1, lat2, lng2, direction, corridor, state, eventId, stateKey) receives the event's primary and secondary points straight from the feed record and passes them through to snapToRoadImmediate(), which builds the URL. Note the order flips: OSRM takes lon,lat while the feeds carry lat,lng.</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>overview=full &amp; geometries=geojson on every call. 10 s timeout (12 s for the via variant).</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Effectively one request per distinct zone geometry, ever. getOSRMCacheKey() rounds both endpoints to 5 decimal places (~1 m) and appends a normalized direction; the result is persisted in the osrm_geometry_cache table, so a repeat of the same zone is served from the database and never re-requested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>{sLon},{sLat};{vLon},{vLat};{eLon},{eLat}</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>OSRM route service v1 (via-point variant)</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Start, an intermediate via point, and end — three coordinates instead of two.</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Used for diversion routes. A plain A→B request returns the shortest path, which for a parallel diversion is usually the main corridor itself — the very road being closed. Forcing the route through a via point on the alternate road makes OSRM return the diversion rather than the highway.</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Same overview=full &amp; geometries=geojson; 12 s timeout.</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>One request per diversion route computed; cached like the 2-point form.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>{n}</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>IBI/511 camera platforms (511PA, DriveNC, AZ511, 511GA, UDOT, NVRoads, 511 Idaho, 511LA, New England 511)</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>A pagination offset. These are DataTables endpoints: POST with body draw=1&amp;start={n}&amp;length=1000.</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>services/camera-adapters.js ibi511Cameras() starts at 0 and advances start by the number of rows actually returned, stopping when it reaches recordsTotal from the response or hits a 20,000 hard ceiling.</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>length 1000 per page; maxima 20,000 rows; 4 attempts per page with 400 ms × attempt backoff.</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Ceil(cameras / 1000) requests per network. The retry-with-backoff exists because under concurrent load — all state adapters firing at once — these hosts intermittently drop a request, and a single silent miss was truncating Georgia at roughly 1,500 of its 4,043 cameras.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>{AccountSid}</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Twilio Programmable SMS</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>The Twilio account identifier embedded in the REST path.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>services/notification-service.js reads process.env.TWILIO_ACCOUNT_SID and TWILIO_AUTH_TOKEN and hands them to the twilio client, which composes the path. Never assembled by hand.</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>TWILIO_ACCOUNT_SID, TWILIO_AUTH_TOKEN, TWILIO_PHONE_NUMBER.</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Outbound only — this ingests no data. One request per SMS sent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>{STATE} / {YEAR}  (resolved)</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD and NHTSA FARS</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Both were templates only because the value is chosen at call time; each resolves to a finite, enumerable set.</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD: services/arnold-geometry-service.js holds a STATE_CODES map of 48 mainland states and a fixed ARNOLD_YEAR constant. FARS: services/crash-data-service.js defaultYears() returns a rolling five-year window ending at (current year − 1).</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>ARNOLD_YEAR = '2019'. FARS window = 2021–2025 as of this compile; it advances by one each January.</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Both sets are now written out individually — see the ARNOLD tab and the five FARS rows on the reference tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr"/>
+      <c r="C8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>NOT FETCHED</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr"/>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>URLs that appear in the code but are never requested — they are emitted for display.</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr"/>
+      <c r="E9" s="10" t="inlineStr"/>
+      <c r="F9" s="10" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>https://api.weather.gov/alerts/{alertId}</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>NOAA / NWS</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Constructed as a permalink on each normalized alert record (the `url` field in services/nws-alerts.js), so a viewer can click through to the official alert. Nothing in the platform ever requests it. The only NWS endpoint actually fetched is https://api.weather.gov/alerts/active.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr"/>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>https://www.grants.gov/search-grants?keywords={oppNumber}</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Grants.gov</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>A human-facing search link attached to each opportunity for click-through. The API calls are search2 and fetchOpportunity.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>